<commit_message>
Fix notification deadlock and update bug reports with BUG-18, BUG-19, BUG-20 details
</commit_message>
<xml_diff>
--- a/bug_report.xlsx
+++ b/bug_report.xlsx
@@ -592,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -613,7 +613,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total bugs found &amp; fixed: 17   |   Smoke tests: PASSED ✅</t>
+          <t>Total bugs found &amp; fixed: 20   |   Smoke tests: PASSED ✅</t>
         </is>
       </c>
     </row>
@@ -1160,92 +1160,92 @@
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="9" t="n">
+      <c r="A21" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>Login — credential validation logic</t>
-        </is>
-      </c>
-      <c r="C21" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D21" s="12" t="inlineStr">
-        <is>
-          <t>routers/auth.py</t>
-        </is>
-      </c>
-      <c r="E21" s="13" t="inlineStr">
-        <is>
-          <t>✅ OK</t>
-        </is>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Booking — notification lock acquisition deadlock</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>BUG-18</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>services/notifications.py</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>🐛 Bug</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>✅ Fixed</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="9" t="n">
+      <c r="A22" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>Rate Limiting — rolling 60-second window</t>
-        </is>
-      </c>
-      <c r="C22" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>services/ratelimit.py</t>
-        </is>
-      </c>
-      <c r="E22" s="13" t="inlineStr">
-        <is>
-          <t>✅ OK</t>
-        </is>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>DateTime — timezone-aware UTC offset stripped instead of converted</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>BUG-19</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>timeutils.py</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>🐛 Bug</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>✅ Fixed</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="9" t="n">
+      <c r="A23" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>Refund Formula — half-up rounding</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D23" s="12" t="inlineStr">
-        <is>
-          <t>services/refunds.py</t>
-        </is>
-      </c>
-      <c r="E23" s="13" t="inlineStr">
-        <is>
-          <t>✅ OK</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Export — include_all scoping bypass exposes other org bookings</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>BUG-20</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>services/export.py</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>🐛 Bug</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>✅ Fixed</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1255,7 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>DateTime UTC — parse &amp; output with +00:00</t>
+          <t>Login — credential validation logic</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
@@ -1265,7 +1265,7 @@
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
-          <t>timeutils.py</t>
+          <t>routers/auth.py</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>Admin Report — includes rooms with zero bookings</t>
+          <t>Rate Limiting — rolling 60-second window</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>routers/admin.py</t>
+          <t>services/ratelimit.py</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>Export CSV — org-scoped, admin-only, UTC timestamps</t>
+          <t>Refund Formula — half-up rounding</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>services/export.py</t>
+          <t>services/refunds.py</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
@@ -1334,6 +1334,36 @@
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Admin Report — includes rooms with zero bookings</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>routers/admin.py</t>
+        </is>
+      </c>
+      <c r="E27" s="13" t="inlineStr">
+        <is>
+          <t>✅ OK</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1354,7 +1384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2034,6 +2064,117 @@
         </is>
       </c>
       <c r="G19" s="20" t="inlineStr">
+        <is>
+          <t>✅ Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="56" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>BUG-18</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="inlineStr">
+        <is>
+          <t>Booking / Concurrency</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>services/notifications.py</t>
+        </is>
+      </c>
+      <c r="D20" s="17" t="inlineStr">
+        <is>
+          <t>L24-36 · notify_created() / notify_cancelled()</t>
+        </is>
+      </c>
+      <c r="E20" s="18" t="inlineStr">
+        <is>
+          <t>Simulated email and audit log locks were acquired in opposite orders in the creation and cancellation paths. Under concurrent load, this could trigger circular-wait deadlocks, freezing the server process.</t>
+        </is>
+      </c>
+      <c r="F20" s="19" t="inlineStr">
+        <is>
+          <t>Unified the locking order in both routines to always acquire _email_lock before _audit_lock.</t>
+        </is>
+      </c>
+      <c r="G20" s="20" t="inlineStr">
+        <is>
+          <t>✅ Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="56" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>BUG-19</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>DateTime</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>timeutils.py</t>
+        </is>
+      </c>
+      <c r="D21" s="17" t="inlineStr">
+        <is>
+          <t>L13 · parse_input_datetime()</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>For timezone-aware datetimes, the offset was stripped (replaced with None) instead of correctly converting the datetime to UTC. This caused incorrect dates and times to be stored for non-UTC input.</t>
+        </is>
+      </c>
+      <c r="F21" s="19" t="inlineStr">
+        <is>
+          <t>Changed the offset check to use astimezone(timezone.utc) before removing tzinfo.</t>
+        </is>
+      </c>
+      <c r="G21" s="20" t="inlineStr">
+        <is>
+          <t>✅ Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="56" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>BUG-20</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>Export / Security</t>
+        </is>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>services/export.py</t>
+        </is>
+      </c>
+      <c r="D22" s="17" t="inlineStr">
+        <is>
+          <t>L44-53 · generate_export()</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="inlineStr">
+        <is>
+          <t>Specifying include_all=true with a room_id bypassed the organization scoping checks, leaking booking details from other organizations.</t>
+        </is>
+      </c>
+      <c r="F22" s="19" t="inlineStr">
+        <is>
+          <t>Enforced room ownership validation checking Room.org_id == org_id before executing raw room queries.</t>
+        </is>
+      </c>
+      <c r="G22" s="20" t="inlineStr">
         <is>
           <t>✅ Fixed</t>
         </is>
@@ -2053,7 +2194,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2107,7 +2248,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C4" s="19" t="inlineStr">
         <is>
@@ -2142,6 +2283,51 @@
       <c r="C6" s="19" t="inlineStr">
         <is>
           <t>BUG-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>app/services/notifications.py</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>BUG-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>app/timeutils.py</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>BUG-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>app/services/export.py</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>BUG-20</t>
         </is>
       </c>
     </row>

</xml_diff>